<commit_message>
Minor Fixes for Room Allotment
</commit_message>
<xml_diff>
--- a/public/files/AdventureEscape.xlsx
+++ b/public/files/AdventureEscape.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\AG_WORK\Automation\JSG-Portal\public\files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2085DC88-AD99-444E-BD55-475C511E8A40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDCFADAC-4046-46D7-8609-620523AAC190}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{5CE65C21-26A1-4929-8A55-619335A4C2C6}"/>
   </bookViews>
@@ -225,9 +225,6 @@
     <t>Viaan Gandhi</t>
   </si>
   <si>
-    <t>Naresh Bhavarlal Shah ( Dhoka)</t>
-  </si>
-  <si>
     <t>D-03</t>
   </si>
   <si>
@@ -327,9 +324,6 @@
     <t>Nivee Kocheta</t>
   </si>
   <si>
-    <t>Hasmukh(Ravee) Chhaganlal oswal</t>
-  </si>
-  <si>
     <t>D-04/05</t>
   </si>
   <si>
@@ -396,9 +390,6 @@
     <t>Davisha Salecha</t>
   </si>
   <si>
-    <t>Jayesh mohanlalji Oswal ( gundesha )</t>
-  </si>
-  <si>
     <t xml:space="preserve">Vaishali Jayesh Oswal </t>
   </si>
   <si>
@@ -462,12 +453,6 @@
     <t>Khush Oswal</t>
   </si>
   <si>
-    <t>Khush shantilal oswal ( Jain)</t>
-  </si>
-  <si>
-    <t>Prisha khush oswal ( Jain)</t>
-  </si>
-  <si>
     <t xml:space="preserve">Kumod Ramesh Kawediya </t>
   </si>
   <si>
@@ -705,9 +690,6 @@
     <t xml:space="preserve">RAJESH  SOGMAL. KHIVSARA </t>
   </si>
   <si>
-    <t xml:space="preserve">KAVITA. RAJESH. KHIVSARA </t>
-  </si>
-  <si>
     <t>Rajesh Lalchand Jain</t>
   </si>
   <si>
@@ -903,12 +885,6 @@
     <t>ISHA</t>
   </si>
   <si>
-    <t>Vipul sumermal lunkad (shah)</t>
-  </si>
-  <si>
-    <t>Mamta vipul lunkad (shah)</t>
-  </si>
-  <si>
     <t>Dhyan</t>
   </si>
   <si>
@@ -940,6 +916,30 @@
   </si>
   <si>
     <t>5 to 8 Yr</t>
+  </si>
+  <si>
+    <t>Naresh Bhavarlal Shah</t>
+  </si>
+  <si>
+    <t>Hasmukh Chhaganlal oswal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jayesh mohanlalji Oswal </t>
+  </si>
+  <si>
+    <t>Khush shantilal oswal</t>
+  </si>
+  <si>
+    <t>Vipul sumermal lunkad</t>
+  </si>
+  <si>
+    <t>Prisha khush oswal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KAVITA RAJESH KHIVSARA </t>
+  </si>
+  <si>
+    <t>Mamta vipul lunkad</t>
   </si>
 </sst>
 </file>
@@ -1605,7 +1605,7 @@
     </row>
     <row r="2" spans="1:38" s="17" customFormat="1" ht="32.4" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="32" t="s">
-        <v>294</v>
+        <v>286</v>
       </c>
       <c r="B2" s="7" t="s">
         <v>0</v>
@@ -1790,16 +1790,16 @@
         <v>36</v>
       </c>
       <c r="X3" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="Y3" s="21" t="s">
-        <v>297</v>
+        <v>289</v>
       </c>
       <c r="Z3" s="21" t="s">
-        <v>298</v>
+        <v>290</v>
       </c>
       <c r="AA3" s="21" t="s">
-        <v>298</v>
+        <v>290</v>
       </c>
       <c r="AB3" s="22">
         <v>2</v>
@@ -1910,10 +1910,10 @@
         <v>#VALUE!</v>
       </c>
       <c r="Z4" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AA4" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AB4" s="22">
         <v>2</v>
@@ -2019,10 +2019,10 @@
         <v>#VALUE!</v>
       </c>
       <c r="Z5" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AA5" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AB5" s="22">
         <v>2</v>
@@ -2130,10 +2130,10 @@
         <v>#VALUE!</v>
       </c>
       <c r="Z6" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AA6" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AB6" s="22">
         <v>2</v>
@@ -2243,7 +2243,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="AA7" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AB7" s="22">
         <v>2</v>
@@ -2277,22 +2277,22 @@
         <v>8087600125</v>
       </c>
       <c r="B8" s="29" t="s">
-        <v>60</v>
+        <v>291</v>
       </c>
       <c r="C8" s="29">
         <v>6</v>
       </c>
       <c r="D8" s="30" t="s">
+        <v>60</v>
+      </c>
+      <c r="E8" s="29" t="s">
         <v>61</v>
-      </c>
-      <c r="E8" s="29" t="s">
-        <v>62</v>
       </c>
       <c r="F8" s="29">
         <v>4</v>
       </c>
       <c r="G8" s="30" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="H8" s="29" t="s">
         <v>36</v>
@@ -2349,10 +2349,10 @@
         <v>#VALUE!</v>
       </c>
       <c r="Z8" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AA8" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AB8" s="22">
         <v>2</v>
@@ -2382,14 +2382,14 @@
         <v>9011090203</v>
       </c>
       <c r="B9" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="C9" s="18" t="s">
         <v>64</v>
       </c>
-      <c r="C9" s="18" t="s">
+      <c r="D9" s="19" t="s">
         <v>65</v>
       </c>
-      <c r="D9" s="19" t="s">
-        <v>66</v>
-      </c>
       <c r="E9" s="18" t="s">
         <v>36</v>
       </c>
@@ -2454,10 +2454,10 @@
         <v>#VALUE!</v>
       </c>
       <c r="Z9" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AA9" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AB9" s="22">
         <v>1</v>
@@ -2492,7 +2492,7 @@
         <v>9820369920</v>
       </c>
       <c r="B10" s="25" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C10" s="25" t="s">
         <v>55</v>
@@ -2564,10 +2564,10 @@
         <v>#VALUE!</v>
       </c>
       <c r="Z10" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AA10" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AB10" s="22">
         <v>1</v>
@@ -2585,7 +2585,7 @@
         <v>3700</v>
       </c>
       <c r="AI10" s="22" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="AJ10" s="22">
         <v>0</v>
@@ -2597,23 +2597,23 @@
         <v>9822011234</v>
       </c>
       <c r="B11" s="29" t="s">
+        <v>68</v>
+      </c>
+      <c r="C11" s="29" t="s">
+        <v>64</v>
+      </c>
+      <c r="D11" s="30" t="s">
+        <v>65</v>
+      </c>
+      <c r="E11" s="29" t="s">
         <v>69</v>
       </c>
-      <c r="C11" s="29" t="s">
-        <v>65</v>
-      </c>
-      <c r="D11" s="30" t="s">
-        <v>66</v>
-      </c>
-      <c r="E11" s="29" t="s">
+      <c r="F11" s="29" t="s">
+        <v>64</v>
+      </c>
+      <c r="G11" s="30" t="s">
         <v>70</v>
       </c>
-      <c r="F11" s="29" t="s">
-        <v>65</v>
-      </c>
-      <c r="G11" s="30" t="s">
-        <v>71</v>
-      </c>
       <c r="H11" s="29" t="s">
         <v>36</v>
       </c>
@@ -2669,10 +2669,10 @@
         <v>#VALUE!</v>
       </c>
       <c r="Z11" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AA11" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AB11" s="22">
         <v>2</v>
@@ -2702,23 +2702,23 @@
         <v>9422301621</v>
       </c>
       <c r="B12" s="18" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C12" s="18">
         <v>3</v>
       </c>
       <c r="D12" s="19" t="s">
+        <v>72</v>
+      </c>
+      <c r="E12" s="18" t="s">
         <v>73</v>
       </c>
-      <c r="E12" s="18" t="s">
+      <c r="F12" s="18" t="s">
         <v>74</v>
       </c>
-      <c r="F12" s="18" t="s">
+      <c r="G12" s="19" t="s">
         <v>75</v>
       </c>
-      <c r="G12" s="19" t="s">
-        <v>76</v>
-      </c>
       <c r="H12" s="18" t="s">
         <v>36</v>
       </c>
@@ -2774,10 +2774,10 @@
         <v>#VALUE!</v>
       </c>
       <c r="Z12" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AA12" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AB12" s="22">
         <v>2</v>
@@ -2814,25 +2814,25 @@
         <v>9850059291</v>
       </c>
       <c r="B13" s="25" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C13" s="25">
         <v>10</v>
       </c>
       <c r="D13" s="26" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E13" s="25" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F13" s="25">
         <v>9</v>
       </c>
       <c r="G13" s="26" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="H13" s="25" t="s">
-        <v>295</v>
+        <v>287</v>
       </c>
       <c r="I13" s="27" t="s">
         <v>36</v>
@@ -2841,10 +2841,10 @@
         <v>#VALUE!</v>
       </c>
       <c r="K13" s="26" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="L13" s="25" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="M13" s="27" t="s">
         <v>36</v>
@@ -2853,7 +2853,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="O13" s="26" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="P13" s="25" t="s">
         <v>36</v>
@@ -2889,7 +2889,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="AA13" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AB13" s="22">
         <v>2</v>
@@ -2927,7 +2927,7 @@
         <v>9561023455</v>
       </c>
       <c r="B14" s="29" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C14" s="29" t="s">
         <v>40</v>
@@ -2936,7 +2936,7 @@
         <v>41</v>
       </c>
       <c r="E14" s="29" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F14" s="29" t="s">
         <v>40</v>
@@ -2999,10 +2999,10 @@
         <v>#VALUE!</v>
       </c>
       <c r="Z14" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AA14" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AB14" s="22">
         <v>2</v>
@@ -3036,7 +3036,7 @@
         <v>8975797500</v>
       </c>
       <c r="B15" s="18" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C15" s="18" t="s">
         <v>55</v>
@@ -3045,7 +3045,7 @@
         <v>56</v>
       </c>
       <c r="E15" s="18" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="F15" s="18" t="s">
         <v>55</v>
@@ -3054,7 +3054,7 @@
         <v>58</v>
       </c>
       <c r="H15" s="18" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="I15" s="20">
         <v>41013</v>
@@ -3063,7 +3063,7 @@
         <v>14</v>
       </c>
       <c r="K15" s="19" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="L15" s="18" t="s">
         <v>36</v>
@@ -3102,7 +3102,7 @@
         <v>36</v>
       </c>
       <c r="X15" s="21" t="s">
-        <v>297</v>
+        <v>289</v>
       </c>
       <c r="Y15" s="21" t="e">
         <v>#VALUE!</v>
@@ -3111,7 +3111,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="AA15" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AB15" s="22">
         <v>2</v>
@@ -3148,25 +3148,25 @@
         <v>9028590888</v>
       </c>
       <c r="B16" s="25" t="s">
+        <v>84</v>
+      </c>
+      <c r="C16" s="25" t="s">
         <v>85</v>
-      </c>
-      <c r="C16" s="25" t="s">
-        <v>86</v>
       </c>
       <c r="D16" s="26" t="s">
         <v>47</v>
       </c>
       <c r="E16" s="25" t="s">
+        <v>86</v>
+      </c>
+      <c r="F16" s="25" t="s">
         <v>87</v>
-      </c>
-      <c r="F16" s="25" t="s">
-        <v>88</v>
       </c>
       <c r="G16" s="26" t="s">
         <v>58</v>
       </c>
       <c r="H16" s="25" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="I16" s="27" t="s">
         <v>36</v>
@@ -3223,7 +3223,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="AA16" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AB16" s="22">
         <v>2</v>
@@ -3243,7 +3243,7 @@
         <v>10200</v>
       </c>
       <c r="AI16" s="22" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="AJ16" s="22">
         <v>0</v>
@@ -3255,7 +3255,7 @@
         <v>7020693176</v>
       </c>
       <c r="B17" s="29" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C17" s="29" t="s">
         <v>40</v>
@@ -3264,7 +3264,7 @@
         <v>41</v>
       </c>
       <c r="E17" s="29" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="F17" s="29" t="s">
         <v>40</v>
@@ -3273,7 +3273,7 @@
         <v>43</v>
       </c>
       <c r="H17" s="29" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="I17" s="31" t="s">
         <v>36</v>
@@ -3330,7 +3330,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="AA17" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AB17" s="22">
         <v>2</v>
@@ -3366,38 +3366,38 @@
         <v>9881766789</v>
       </c>
       <c r="B18" s="18" t="s">
-        <v>94</v>
+        <v>292</v>
       </c>
       <c r="C18" s="18">
         <v>9</v>
       </c>
       <c r="D18" s="19" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="E18" s="18" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="F18" s="18">
         <v>8</v>
       </c>
       <c r="G18" s="19" t="s">
+        <v>95</v>
+      </c>
+      <c r="H18" s="18" t="s">
+        <v>96</v>
+      </c>
+      <c r="I18" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="J18" s="18" t="e">
+        <v>#VALUE!</v>
+      </c>
+      <c r="K18" s="19" t="s">
+        <v>95</v>
+      </c>
+      <c r="L18" s="18" t="s">
         <v>97</v>
       </c>
-      <c r="H18" s="18" t="s">
-        <v>98</v>
-      </c>
-      <c r="I18" s="20" t="s">
-        <v>36</v>
-      </c>
-      <c r="J18" s="18" t="e">
-        <v>#VALUE!</v>
-      </c>
-      <c r="K18" s="19" t="s">
-        <v>97</v>
-      </c>
-      <c r="L18" s="18" t="s">
-        <v>99</v>
-      </c>
       <c r="M18" s="20" t="s">
         <v>36</v>
       </c>
@@ -3405,7 +3405,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="O18" s="19" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="P18" s="18" t="s">
         <v>36</v>
@@ -3441,7 +3441,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="AA18" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AB18" s="22">
         <v>2</v>
@@ -3478,26 +3478,26 @@
         <v>9960429494</v>
       </c>
       <c r="B19" s="25" t="s">
+        <v>98</v>
+      </c>
+      <c r="C19" s="25" t="s">
+        <v>64</v>
+      </c>
+      <c r="D19" s="26" t="s">
+        <v>65</v>
+      </c>
+      <c r="E19" s="25" t="s">
+        <v>99</v>
+      </c>
+      <c r="F19" s="25" t="s">
+        <v>64</v>
+      </c>
+      <c r="G19" s="26" t="s">
+        <v>70</v>
+      </c>
+      <c r="H19" s="25" t="s">
         <v>100</v>
       </c>
-      <c r="C19" s="25" t="s">
-        <v>65</v>
-      </c>
-      <c r="D19" s="26" t="s">
-        <v>66</v>
-      </c>
-      <c r="E19" s="25" t="s">
-        <v>101</v>
-      </c>
-      <c r="F19" s="25" t="s">
-        <v>65</v>
-      </c>
-      <c r="G19" s="26" t="s">
-        <v>71</v>
-      </c>
-      <c r="H19" s="25" t="s">
-        <v>102</v>
-      </c>
       <c r="I19" s="27" t="s">
         <v>36</v>
       </c>
@@ -3505,7 +3505,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="K19" s="26" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="L19" s="25" t="s">
         <v>36</v>
@@ -3553,7 +3553,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="AA19" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AB19" s="22">
         <v>2</v>
@@ -3581,7 +3581,7 @@
         <v>0</v>
       </c>
       <c r="AK19" s="3" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
     </row>
     <row r="20" spans="1:38" s="17" customFormat="1" ht="16" x14ac:dyDescent="0.35">
@@ -3589,16 +3589,16 @@
         <v>8668533098</v>
       </c>
       <c r="B20" s="29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="C20" s="29">
         <v>7</v>
       </c>
       <c r="D20" s="30" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="E20" s="29" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="F20" s="29">
         <v>5</v>
@@ -3661,10 +3661,10 @@
         <v>#VALUE!</v>
       </c>
       <c r="Z20" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AA20" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AB20" s="22">
         <v>2</v>
@@ -3700,25 +3700,25 @@
         <v>8766422772</v>
       </c>
       <c r="B21" s="18" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C21" s="18">
         <v>9</v>
       </c>
       <c r="D21" s="19" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="E21" s="18" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="F21" s="18">
         <v>8</v>
       </c>
       <c r="G21" s="19" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="H21" s="18" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="I21" s="20" t="s">
         <v>36</v>
@@ -3727,20 +3727,20 @@
         <v>#VALUE!</v>
       </c>
       <c r="K21" s="19" t="s">
+        <v>93</v>
+      </c>
+      <c r="L21" s="18" t="s">
+        <v>108</v>
+      </c>
+      <c r="M21" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="N21" s="18" t="e">
+        <v>#VALUE!</v>
+      </c>
+      <c r="O21" s="19" t="s">
         <v>95</v>
       </c>
-      <c r="L21" s="18" t="s">
-        <v>110</v>
-      </c>
-      <c r="M21" s="20" t="s">
-        <v>36</v>
-      </c>
-      <c r="N21" s="18" t="e">
-        <v>#VALUE!</v>
-      </c>
-      <c r="O21" s="19" t="s">
-        <v>97</v>
-      </c>
       <c r="P21" s="18" t="s">
         <v>36</v>
       </c>
@@ -3775,7 +3775,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="AA21" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AB21" s="22">
         <v>2</v>
@@ -3812,47 +3812,47 @@
         <v>9028988457</v>
       </c>
       <c r="B22" s="25" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="C22" s="25">
         <v>5</v>
       </c>
       <c r="D22" s="26" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E22" s="25" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="F22" s="25">
         <v>3</v>
       </c>
       <c r="G22" s="26" t="s">
+        <v>112</v>
+      </c>
+      <c r="H22" s="25" t="s">
+        <v>113</v>
+      </c>
+      <c r="I22" s="27" t="s">
+        <v>36</v>
+      </c>
+      <c r="J22" s="25" t="e">
+        <v>#VALUE!</v>
+      </c>
+      <c r="K22" s="26" t="s">
+        <v>110</v>
+      </c>
+      <c r="L22" s="25" t="s">
         <v>114</v>
       </c>
-      <c r="H22" s="25" t="s">
-        <v>115</v>
-      </c>
-      <c r="I22" s="27" t="s">
-        <v>36</v>
-      </c>
-      <c r="J22" s="25" t="e">
-        <v>#VALUE!</v>
-      </c>
-      <c r="K22" s="26" t="s">
+      <c r="M22" s="27" t="s">
+        <v>36</v>
+      </c>
+      <c r="N22" s="25" t="e">
+        <v>#VALUE!</v>
+      </c>
+      <c r="O22" s="26" t="s">
         <v>112</v>
       </c>
-      <c r="L22" s="25" t="s">
-        <v>116</v>
-      </c>
-      <c r="M22" s="27" t="s">
-        <v>36</v>
-      </c>
-      <c r="N22" s="25" t="e">
-        <v>#VALUE!</v>
-      </c>
-      <c r="O22" s="26" t="s">
-        <v>114</v>
-      </c>
       <c r="P22" s="25" t="s">
         <v>36</v>
       </c>
@@ -3887,7 +3887,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="AA22" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AB22" s="22">
         <v>2</v>
@@ -3923,16 +3923,16 @@
         <v>9822211123</v>
       </c>
       <c r="B23" s="29" t="s">
-        <v>117</v>
+        <v>293</v>
       </c>
       <c r="C23" s="29">
         <v>7</v>
       </c>
       <c r="D23" s="30" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="E23" s="29" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="F23" s="29">
         <v>5</v>
@@ -3995,10 +3995,10 @@
         <v>#VALUE!</v>
       </c>
       <c r="Z23" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AA23" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AB23" s="22">
         <v>2</v>
@@ -4034,7 +4034,7 @@
         <v>9890377803</v>
       </c>
       <c r="B24" s="18" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="C24" s="18">
         <v>4</v>
@@ -4043,7 +4043,7 @@
         <v>31</v>
       </c>
       <c r="E24" s="18" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="F24" s="18">
         <v>2</v>
@@ -4052,7 +4052,7 @@
         <v>33</v>
       </c>
       <c r="H24" s="18" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="I24" s="20" t="s">
         <v>36</v>
@@ -4109,7 +4109,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="AA24" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AB24" s="22">
         <v>2</v>
@@ -4148,7 +4148,7 @@
         <v>9822519391</v>
       </c>
       <c r="B25" s="25" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="C25" s="25" t="s">
         <v>55</v>
@@ -4157,7 +4157,7 @@
         <v>56</v>
       </c>
       <c r="E25" s="25" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="F25" s="25" t="s">
         <v>55</v>
@@ -4220,10 +4220,10 @@
         <v>#VALUE!</v>
       </c>
       <c r="Z25" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AA25" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AB25" s="22">
         <v>2</v>
@@ -4257,16 +4257,16 @@
         <v>9822094100</v>
       </c>
       <c r="B26" s="29" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="C26" s="29">
         <v>7</v>
       </c>
       <c r="D26" s="30" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="E26" s="29" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="F26" s="29">
         <v>5</v>
@@ -4329,10 +4329,10 @@
         <v>#VALUE!</v>
       </c>
       <c r="Z26" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AA26" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AB26" s="22">
         <v>2</v>
@@ -4368,25 +4368,25 @@
         <v>9890265366</v>
       </c>
       <c r="B27" s="18" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="C27" s="18">
         <v>6</v>
       </c>
       <c r="D27" s="19" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E27" s="18" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="F27" s="18">
         <v>4</v>
       </c>
       <c r="G27" s="19" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="H27" s="18" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="I27" s="20" t="s">
         <v>36</v>
@@ -4395,7 +4395,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="K27" s="19" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="L27" s="18" t="s">
         <v>36</v>
@@ -4443,7 +4443,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="AA27" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AB27" s="22">
         <v>2</v>
@@ -4480,50 +4480,50 @@
         <v>9372550100</v>
       </c>
       <c r="B28" s="25" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="C28" s="25">
         <v>6</v>
       </c>
       <c r="D28" s="26" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E28" s="25" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="F28" s="25">
         <v>4</v>
       </c>
       <c r="G28" s="26" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="H28" s="25" t="s">
+        <v>128</v>
+      </c>
+      <c r="I28" s="27" t="s">
+        <v>36</v>
+      </c>
+      <c r="J28" s="25" t="e">
+        <v>#VALUE!</v>
+      </c>
+      <c r="K28" s="26" t="s">
+        <v>60</v>
+      </c>
+      <c r="L28" s="25" t="s">
+        <v>129</v>
+      </c>
+      <c r="M28" s="27" t="s">
+        <v>36</v>
+      </c>
+      <c r="N28" s="25" t="e">
+        <v>#VALUE!</v>
+      </c>
+      <c r="O28" s="26" t="s">
+        <v>130</v>
+      </c>
+      <c r="P28" s="25" t="s">
         <v>131</v>
       </c>
-      <c r="I28" s="27" t="s">
-        <v>36</v>
-      </c>
-      <c r="J28" s="25" t="e">
-        <v>#VALUE!</v>
-      </c>
-      <c r="K28" s="26" t="s">
-        <v>61</v>
-      </c>
-      <c r="L28" s="25" t="s">
-        <v>132</v>
-      </c>
-      <c r="M28" s="27" t="s">
-        <v>36</v>
-      </c>
-      <c r="N28" s="25" t="e">
-        <v>#VALUE!</v>
-      </c>
-      <c r="O28" s="26" t="s">
-        <v>133</v>
-      </c>
-      <c r="P28" s="25" t="s">
-        <v>134</v>
-      </c>
       <c r="Q28" s="27" t="s">
         <v>36</v>
       </c>
@@ -4531,7 +4531,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="S28" s="25" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="T28" s="25" t="s">
         <v>36</v>
@@ -4555,7 +4555,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="AA28" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AB28" s="22">
         <v>2</v>
@@ -4591,25 +4591,25 @@
         <v>9765576667</v>
       </c>
       <c r="B29" s="29" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="C29" s="29" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D29" s="30" t="s">
         <v>31</v>
       </c>
       <c r="E29" s="29" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="F29" s="29" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G29" s="30" t="s">
         <v>33</v>
       </c>
       <c r="H29" s="29" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="I29" s="31" t="s">
         <v>36</v>
@@ -4666,7 +4666,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="AA29" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AB29" s="22">
         <v>2</v>
@@ -4700,7 +4700,7 @@
         <v>9028661666</v>
       </c>
       <c r="B30" s="18" t="s">
-        <v>139</v>
+        <v>294</v>
       </c>
       <c r="C30" s="18" t="s">
         <v>55</v>
@@ -4709,7 +4709,7 @@
         <v>56</v>
       </c>
       <c r="E30" s="18" t="s">
-        <v>140</v>
+        <v>296</v>
       </c>
       <c r="F30" s="18" t="s">
         <v>55</v>
@@ -4772,10 +4772,10 @@
         <v>#VALUE!</v>
       </c>
       <c r="Z30" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AA30" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AB30" s="22">
         <v>2</v>
@@ -4793,7 +4793,7 @@
         <v>7400</v>
       </c>
       <c r="AI30" s="22" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="AJ30" s="22">
         <v>0</v>
@@ -4808,25 +4808,25 @@
         <v>9503044333</v>
       </c>
       <c r="B31" s="25" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="C31" s="25" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="D31" s="26" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="E31" s="25" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="F31" s="25">
         <v>6</v>
       </c>
       <c r="G31" s="26" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
       <c r="H31" s="25" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="I31" s="27" t="s">
         <v>36</v>
@@ -4835,10 +4835,10 @@
         <v>#VALUE!</v>
       </c>
       <c r="K31" s="26" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="L31" s="25" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="M31" s="27" t="s">
         <v>36</v>
@@ -4847,7 +4847,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="O31" s="26" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
       <c r="P31" s="25" t="s">
         <v>36</v>
@@ -4883,7 +4883,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="AA31" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AB31" s="22">
         <v>2</v>
@@ -4911,7 +4911,7 @@
         <v>0</v>
       </c>
       <c r="AK31" s="3" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
     </row>
     <row r="32" spans="1:38" s="17" customFormat="1" ht="16" x14ac:dyDescent="0.35">
@@ -4919,25 +4919,25 @@
         <v>9545075151</v>
       </c>
       <c r="B32" s="29" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="C32" s="29">
         <v>11</v>
       </c>
       <c r="D32" s="30" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="E32" s="29" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="F32" s="29">
         <v>10</v>
       </c>
       <c r="G32" s="30" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H32" s="29" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="I32" s="31" t="s">
         <v>36</v>
@@ -4946,7 +4946,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="K32" s="30" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="L32" s="29" t="s">
         <v>36</v>
@@ -4994,7 +4994,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="AA32" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AB32" s="22">
         <v>2</v>
@@ -5032,7 +5032,7 @@
         <v>9130128128</v>
       </c>
       <c r="B33" s="18" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
       <c r="C33" s="18">
         <v>8</v>
@@ -5041,7 +5041,7 @@
         <v>47</v>
       </c>
       <c r="E33" s="18" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
       <c r="F33" s="18">
         <v>7</v>
@@ -5050,7 +5050,7 @@
         <v>49</v>
       </c>
       <c r="H33" s="18" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="I33" s="20" t="s">
         <v>36</v>
@@ -5107,7 +5107,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="AA33" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AB33" s="22">
         <v>2</v>
@@ -5144,25 +5144,25 @@
         <v>9028483439</v>
       </c>
       <c r="B34" s="25" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
       <c r="C34" s="25">
         <v>6</v>
       </c>
       <c r="D34" s="26" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E34" s="25" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
       <c r="F34" s="25">
         <v>4</v>
       </c>
       <c r="G34" s="26" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="H34" s="25" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="I34" s="27" t="s">
         <v>36</v>
@@ -5171,7 +5171,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="K34" s="26" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="L34" s="25" t="s">
         <v>36</v>
@@ -5219,7 +5219,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="AA34" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AB34" s="22">
         <v>2</v>
@@ -5255,23 +5255,23 @@
         <v>9422008832</v>
       </c>
       <c r="B35" s="29" t="s">
-        <v>158</v>
+        <v>153</v>
       </c>
       <c r="C35" s="29">
         <v>3</v>
       </c>
       <c r="D35" s="30" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E35" s="29" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="F35" s="29" t="s">
+        <v>74</v>
+      </c>
+      <c r="G35" s="30" t="s">
         <v>75</v>
       </c>
-      <c r="G35" s="30" t="s">
-        <v>76</v>
-      </c>
       <c r="H35" s="29" t="s">
         <v>36</v>
       </c>
@@ -5327,10 +5327,10 @@
         <v>#VALUE!</v>
       </c>
       <c r="Z35" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AA35" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AB35" s="22">
         <v>2</v>
@@ -5366,22 +5366,22 @@
         <v>7972483559</v>
       </c>
       <c r="B36" s="18" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="C36" s="18">
         <v>11</v>
       </c>
       <c r="D36" s="19" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="E36" s="18" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
       <c r="F36" s="18">
         <v>10</v>
       </c>
       <c r="G36" s="19" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H36" s="18" t="s">
         <v>36</v>
@@ -5438,10 +5438,10 @@
         <v>#VALUE!</v>
       </c>
       <c r="Z36" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AA36" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AB36" s="22">
         <v>2</v>
@@ -5478,16 +5478,16 @@
         <v>8087549644</v>
       </c>
       <c r="B37" s="25" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="C37" s="25">
         <v>7</v>
       </c>
       <c r="D37" s="26" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="E37" s="25" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="F37" s="25">
         <v>5</v>
@@ -5496,7 +5496,7 @@
         <v>33</v>
       </c>
       <c r="H37" s="25" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
       <c r="I37" s="27" t="s">
         <v>36</v>
@@ -5553,7 +5553,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="AA37" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AB37" s="22">
         <v>2</v>
@@ -5589,25 +5589,25 @@
         <v>9860171721</v>
       </c>
       <c r="B38" s="29" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="C38" s="29" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D38" s="30" t="s">
         <v>31</v>
       </c>
       <c r="E38" s="29" t="s">
-        <v>167</v>
+        <v>162</v>
       </c>
       <c r="F38" s="29" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G38" s="30" t="s">
         <v>33</v>
       </c>
       <c r="H38" s="29" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="I38" s="31" t="s">
         <v>36</v>
@@ -5664,7 +5664,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="AA38" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AB38" s="22">
         <v>2</v>
@@ -5700,14 +5700,14 @@
         <v>8446535244</v>
       </c>
       <c r="B39" s="18" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="C39" s="18" t="s">
+        <v>64</v>
+      </c>
+      <c r="D39" s="19" t="s">
         <v>65</v>
       </c>
-      <c r="D39" s="19" t="s">
-        <v>66</v>
-      </c>
       <c r="E39" s="18" t="s">
         <v>36</v>
       </c>
@@ -5772,10 +5772,10 @@
         <v>#VALUE!</v>
       </c>
       <c r="Z39" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AA39" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AB39" s="22">
         <v>1</v>
@@ -5810,7 +5810,7 @@
         <v>9422546094</v>
       </c>
       <c r="B40" s="25" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="C40" s="25">
         <v>8</v>
@@ -5819,7 +5819,7 @@
         <v>47</v>
       </c>
       <c r="E40" s="25" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="F40" s="25">
         <v>7</v>
@@ -5828,7 +5828,7 @@
         <v>49</v>
       </c>
       <c r="H40" s="25" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
       <c r="I40" s="27" t="s">
         <v>36</v>
@@ -5840,7 +5840,7 @@
         <v>49</v>
       </c>
       <c r="L40" s="25" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="M40" s="27" t="s">
         <v>36</v>
@@ -5885,7 +5885,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="AA40" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AB40" s="22">
         <v>2</v>
@@ -5919,7 +5919,7 @@
         <v>9420277778</v>
       </c>
       <c r="B41" s="29" t="s">
-        <v>174</v>
+        <v>169</v>
       </c>
       <c r="C41" s="29" t="s">
         <v>55</v>
@@ -5928,7 +5928,7 @@
         <v>56</v>
       </c>
       <c r="E41" s="29" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
       <c r="F41" s="29" t="s">
         <v>55</v>
@@ -5937,7 +5937,7 @@
         <v>58</v>
       </c>
       <c r="H41" s="29" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
       <c r="I41" s="31" t="s">
         <v>36</v>
@@ -5994,7 +5994,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="AA41" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AB41" s="22">
         <v>2</v>
@@ -6028,25 +6028,25 @@
         <v>9371234228</v>
       </c>
       <c r="B42" s="18" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="C42" s="18">
         <v>6</v>
       </c>
       <c r="D42" s="19" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E42" s="18" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
       <c r="F42" s="18">
         <v>4</v>
       </c>
       <c r="G42" s="19" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="H42" s="18" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="I42" s="20" t="s">
         <v>36</v>
@@ -6055,10 +6055,10 @@
         <v>#VALUE!</v>
       </c>
       <c r="K42" s="19" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="L42" s="18" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
       <c r="M42" s="20" t="s">
         <v>36</v>
@@ -6067,7 +6067,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="O42" s="19" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="P42" s="18" t="s">
         <v>36</v>
@@ -6103,7 +6103,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="AA42" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AB42" s="22">
         <v>2</v>
@@ -6140,25 +6140,25 @@
         <v>8956774747</v>
       </c>
       <c r="B43" s="25" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="C43" s="25" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D43" s="26" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E43" s="25" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
       <c r="F43" s="25" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G43" s="26" t="s">
         <v>43</v>
       </c>
       <c r="H43" s="25" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="I43" s="27" t="s">
         <v>36</v>
@@ -6170,7 +6170,7 @@
         <v>43</v>
       </c>
       <c r="L43" s="25" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
       <c r="M43" s="27" t="s">
         <v>36</v>
@@ -6215,7 +6215,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="AA43" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AB43" s="22">
         <v>2</v>
@@ -6251,7 +6251,7 @@
         <v>8446735443</v>
       </c>
       <c r="B44" s="29" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
       <c r="C44" s="29">
         <v>8</v>
@@ -6260,7 +6260,7 @@
         <v>47</v>
       </c>
       <c r="E44" s="29" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="F44" s="29">
         <v>7</v>
@@ -6269,7 +6269,7 @@
         <v>49</v>
       </c>
       <c r="H44" s="29" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="I44" s="31" t="s">
         <v>36</v>
@@ -6326,7 +6326,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="AA44" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AB44" s="22">
         <v>2</v>
@@ -6364,22 +6364,22 @@
         <v>9637898033</v>
       </c>
       <c r="B45" s="18" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
       <c r="C45" s="18" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D45" s="19" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E45" s="18" t="s">
-        <v>188</v>
+        <v>183</v>
       </c>
       <c r="F45" s="18" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G45" s="19" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
       <c r="H45" s="18" t="s">
         <v>36</v>
@@ -6436,10 +6436,10 @@
         <v>#VALUE!</v>
       </c>
       <c r="Z45" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AA45" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AB45" s="22">
         <v>2</v>
@@ -6474,22 +6474,22 @@
         <v>9326243737</v>
       </c>
       <c r="B46" s="25" t="s">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="C46" s="25" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="D46" s="26" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="E46" s="25" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
       <c r="F46" s="25">
         <v>6</v>
       </c>
       <c r="G46" s="26" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
       <c r="H46" s="25" t="s">
         <v>36</v>
@@ -6546,10 +6546,10 @@
         <v>#VALUE!</v>
       </c>
       <c r="Z46" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AA46" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AB46" s="22">
         <v>2</v>
@@ -6581,22 +6581,22 @@
         <v>9850140222</v>
       </c>
       <c r="B47" s="29" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
       <c r="C47" s="29" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D47" s="30" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="E47" s="29" t="s">
-        <v>193</v>
+        <v>188</v>
       </c>
       <c r="F47" s="29" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G47" s="30" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
       <c r="H47" s="29" t="s">
         <v>36</v>
@@ -6653,10 +6653,10 @@
         <v>#VALUE!</v>
       </c>
       <c r="Z47" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AA47" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AB47" s="22">
         <v>2</v>
@@ -6690,25 +6690,25 @@
         <v>9011100000</v>
       </c>
       <c r="B48" s="18" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="C48" s="18">
         <v>11</v>
       </c>
       <c r="D48" s="19" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="E48" s="18" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
       <c r="F48" s="18">
         <v>10</v>
       </c>
       <c r="G48" s="19" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H48" s="18" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="I48" s="20" t="s">
         <v>36</v>
@@ -6717,7 +6717,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="K48" s="19" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="L48" s="18" t="s">
         <v>36</v>
@@ -6765,7 +6765,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="AA48" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AB48" s="22">
         <v>2</v>
@@ -6802,25 +6802,25 @@
         <v>7798983029</v>
       </c>
       <c r="B49" s="25" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="C49" s="25">
         <v>2</v>
       </c>
       <c r="D49" s="26" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="E49" s="25" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
       <c r="F49" s="25">
         <v>1</v>
       </c>
       <c r="G49" s="26" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="H49" s="25" t="s">
-        <v>199</v>
+        <v>194</v>
       </c>
       <c r="I49" s="27" t="s">
         <v>36</v>
@@ -6829,10 +6829,10 @@
         <v>#VALUE!</v>
       </c>
       <c r="K49" s="26" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="L49" s="25" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
       <c r="M49" s="27" t="s">
         <v>36</v>
@@ -6841,7 +6841,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="O49" s="26" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="P49" s="25" t="s">
         <v>36</v>
@@ -6877,7 +6877,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="AA49" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AB49" s="22">
         <v>2</v>
@@ -6911,22 +6911,22 @@
         <v>9822450288</v>
       </c>
       <c r="B50" s="29" t="s">
-        <v>201</v>
+        <v>196</v>
       </c>
       <c r="C50" s="29">
         <v>5</v>
       </c>
       <c r="D50" s="30" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E50" s="29" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
       <c r="F50" s="29">
         <v>3</v>
       </c>
       <c r="G50" s="30" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="H50" s="29" t="s">
         <v>36</v>
@@ -6983,10 +6983,10 @@
         <v>#VALUE!</v>
       </c>
       <c r="Z50" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AA50" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AB50" s="22">
         <v>2</v>
@@ -7022,7 +7022,7 @@
         <v>8668744545</v>
       </c>
       <c r="B51" s="18" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
       <c r="C51" s="18">
         <v>4</v>
@@ -7031,7 +7031,7 @@
         <v>31</v>
       </c>
       <c r="E51" s="18" t="s">
-        <v>204</v>
+        <v>199</v>
       </c>
       <c r="F51" s="18">
         <v>2</v>
@@ -7040,7 +7040,7 @@
         <v>33</v>
       </c>
       <c r="H51" s="18" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
       <c r="I51" s="20" t="s">
         <v>36</v>
@@ -7097,7 +7097,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="AA51" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AB51" s="22">
         <v>2</v>
@@ -7136,7 +7136,7 @@
         <v>9371093117</v>
       </c>
       <c r="B52" s="25" t="s">
-        <v>206</v>
+        <v>201</v>
       </c>
       <c r="C52" s="25" t="s">
         <v>40</v>
@@ -7145,7 +7145,7 @@
         <v>41</v>
       </c>
       <c r="E52" s="25" t="s">
-        <v>207</v>
+        <v>202</v>
       </c>
       <c r="F52" s="25" t="s">
         <v>40</v>
@@ -7208,10 +7208,10 @@
         <v>#VALUE!</v>
       </c>
       <c r="Z52" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AA52" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AB52" s="22">
         <v>2</v>
@@ -7245,13 +7245,13 @@
         <v>7276426863</v>
       </c>
       <c r="B53" s="29" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
       <c r="C53" s="29" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D53" s="30" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="E53" s="29" t="s">
         <v>36</v>
@@ -7317,10 +7317,10 @@
         <v>#VALUE!</v>
       </c>
       <c r="Z53" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AA53" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AB53" s="22">
         <v>1</v>
@@ -7342,13 +7342,13 @@
         <v>3700</v>
       </c>
       <c r="AI53" s="22" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
       <c r="AJ53" s="22">
         <v>0</v>
       </c>
       <c r="AK53" s="3" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
     </row>
     <row r="54" spans="1:38" s="17" customFormat="1" x14ac:dyDescent="0.35">
@@ -7356,25 +7356,25 @@
         <v>9822251329</v>
       </c>
       <c r="B54" s="18" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="C54" s="18">
         <v>2</v>
       </c>
       <c r="D54" s="19" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="E54" s="18" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
       <c r="F54" s="18">
         <v>1</v>
       </c>
       <c r="G54" s="19" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="H54" s="18" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="I54" s="20" t="s">
         <v>36</v>
@@ -7383,7 +7383,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="K54" s="19" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="L54" s="18" t="s">
         <v>36</v>
@@ -7431,7 +7431,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="AA54" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AB54" s="22">
         <v>2</v>
@@ -7466,25 +7466,25 @@
         <v>9423205257</v>
       </c>
       <c r="B55" s="25" t="s">
-        <v>214</v>
+        <v>209</v>
       </c>
       <c r="C55" s="25">
         <v>6</v>
       </c>
       <c r="D55" s="26" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="E55" s="25" t="s">
-        <v>215</v>
+        <v>210</v>
       </c>
       <c r="F55" s="25">
         <v>4</v>
       </c>
       <c r="G55" s="26" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="H55" s="25" t="s">
-        <v>216</v>
+        <v>211</v>
       </c>
       <c r="I55" s="27" t="s">
         <v>36</v>
@@ -7493,10 +7493,10 @@
         <v>#VALUE!</v>
       </c>
       <c r="K55" s="26" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="L55" s="25" t="s">
-        <v>217</v>
+        <v>212</v>
       </c>
       <c r="M55" s="27" t="s">
         <v>36</v>
@@ -7505,7 +7505,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="O55" s="26" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="P55" s="25" t="s">
         <v>36</v>
@@ -7541,7 +7541,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="AA55" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AB55" s="22">
         <v>2</v>
@@ -7571,7 +7571,7 @@
         <v>0</v>
       </c>
       <c r="AK55" s="3" t="s">
-        <v>218</v>
+        <v>213</v>
       </c>
     </row>
     <row r="56" spans="1:38" s="17" customFormat="1" ht="16" x14ac:dyDescent="0.35">
@@ -7579,23 +7579,23 @@
         <v>9423217191</v>
       </c>
       <c r="B56" s="29" t="s">
-        <v>219</v>
+        <v>214</v>
       </c>
       <c r="C56" s="29">
         <v>3</v>
       </c>
       <c r="D56" s="30" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E56" s="29" t="s">
-        <v>220</v>
+        <v>297</v>
       </c>
       <c r="F56" s="29" t="s">
+        <v>74</v>
+      </c>
+      <c r="G56" s="30" t="s">
         <v>75</v>
       </c>
-      <c r="G56" s="30" t="s">
-        <v>76</v>
-      </c>
       <c r="H56" s="29" t="s">
         <v>36</v>
       </c>
@@ -7651,10 +7651,10 @@
         <v>#VALUE!</v>
       </c>
       <c r="Z56" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AA56" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AB56" s="22">
         <v>2</v>
@@ -7690,23 +7690,23 @@
         <v>9175705152</v>
       </c>
       <c r="B57" s="18" t="s">
-        <v>221</v>
+        <v>215</v>
       </c>
       <c r="C57" s="18">
         <v>3</v>
       </c>
       <c r="D57" s="19" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E57" s="18" t="s">
-        <v>222</v>
+        <v>216</v>
       </c>
       <c r="F57" s="18" t="s">
+        <v>74</v>
+      </c>
+      <c r="G57" s="19" t="s">
         <v>75</v>
       </c>
-      <c r="G57" s="19" t="s">
-        <v>76</v>
-      </c>
       <c r="H57" s="18" t="s">
         <v>36</v>
       </c>
@@ -7762,10 +7762,10 @@
         <v>#VALUE!</v>
       </c>
       <c r="Z57" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AA57" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AB57" s="22">
         <v>2</v>
@@ -7804,25 +7804,25 @@
         <v>9158095026</v>
       </c>
       <c r="B58" s="25" t="s">
-        <v>224</v>
+        <v>218</v>
       </c>
       <c r="C58" s="25" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="D58" s="26" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="E58" s="25" t="s">
-        <v>223</v>
+        <v>217</v>
       </c>
       <c r="F58" s="25">
         <v>6</v>
       </c>
       <c r="G58" s="26" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
       <c r="H58" s="25" t="s">
-        <v>225</v>
+        <v>219</v>
       </c>
       <c r="I58" s="27" t="s">
         <v>36</v>
@@ -7831,10 +7831,10 @@
         <v>#VALUE!</v>
       </c>
       <c r="K58" s="26" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
       <c r="L58" s="25" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
       <c r="M58" s="27" t="s">
         <v>36</v>
@@ -7843,7 +7843,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="O58" s="26" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
       <c r="P58" s="25" t="s">
         <v>36</v>
@@ -7879,7 +7879,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="AA58" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AB58" s="22">
         <v>2</v>
@@ -7915,25 +7915,25 @@
         <v>9373002007</v>
       </c>
       <c r="B59" s="29" t="s">
-        <v>227</v>
+        <v>221</v>
       </c>
       <c r="C59" s="29" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="D59" s="30" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="E59" s="29" t="s">
-        <v>228</v>
+        <v>222</v>
       </c>
       <c r="F59" s="29">
         <v>6</v>
       </c>
       <c r="G59" s="30" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
       <c r="H59" s="29" t="s">
-        <v>229</v>
+        <v>223</v>
       </c>
       <c r="I59" s="31" t="s">
         <v>36</v>
@@ -7942,10 +7942,10 @@
         <v>#VALUE!</v>
       </c>
       <c r="K59" s="30" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="L59" s="29" t="s">
-        <v>230</v>
+        <v>224</v>
       </c>
       <c r="M59" s="31" t="s">
         <v>36</v>
@@ -7954,7 +7954,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="O59" s="30" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
       <c r="P59" s="29" t="s">
         <v>36</v>
@@ -7990,7 +7990,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="AA59" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AB59" s="22">
         <v>2</v>
@@ -8022,22 +8022,22 @@
         <v>7972220732</v>
       </c>
       <c r="B60" s="18" t="s">
-        <v>231</v>
+        <v>225</v>
       </c>
       <c r="C60" s="18">
         <v>6</v>
       </c>
       <c r="D60" s="19" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E60" s="18" t="s">
-        <v>232</v>
+        <v>226</v>
       </c>
       <c r="F60" s="18">
         <v>4</v>
       </c>
       <c r="G60" s="19" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="H60" s="18" t="s">
         <v>36</v>
@@ -8094,10 +8094,10 @@
         <v>#VALUE!</v>
       </c>
       <c r="Z60" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AA60" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AB60" s="22">
         <v>2</v>
@@ -8132,25 +8132,25 @@
         <v>9823162182</v>
       </c>
       <c r="B61" s="25" t="s">
-        <v>233</v>
+        <v>227</v>
       </c>
       <c r="C61" s="25">
         <v>2</v>
       </c>
       <c r="D61" s="26" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="E61" s="25" t="s">
-        <v>234</v>
+        <v>228</v>
       </c>
       <c r="F61" s="25">
         <v>1</v>
       </c>
       <c r="G61" s="26" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="H61" s="25" t="s">
-        <v>235</v>
+        <v>229</v>
       </c>
       <c r="I61" s="27" t="s">
         <v>36</v>
@@ -8159,7 +8159,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="K61" s="26" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="L61" s="25" t="s">
         <v>36</v>
@@ -8207,7 +8207,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="AA61" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AB61" s="22">
         <v>2</v>
@@ -8241,19 +8241,19 @@
         <v>9823095979</v>
       </c>
       <c r="B62" s="29" t="s">
-        <v>236</v>
+        <v>230</v>
       </c>
       <c r="C62" s="29" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D62" s="30" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="E62" s="29" t="s">
-        <v>237</v>
+        <v>231</v>
       </c>
       <c r="F62" s="29" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G62" s="30" t="s">
         <v>49</v>
@@ -8313,10 +8313,10 @@
         <v>#VALUE!</v>
       </c>
       <c r="Z62" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AA62" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AB62" s="22">
         <v>2</v>
@@ -8352,25 +8352,25 @@
         <v>9421009818</v>
       </c>
       <c r="B63" s="18" t="s">
-        <v>238</v>
+        <v>232</v>
       </c>
       <c r="C63" s="18" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D63" s="19" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E63" s="18" t="s">
-        <v>239</v>
+        <v>233</v>
       </c>
       <c r="F63" s="18">
         <v>9</v>
       </c>
       <c r="G63" s="19" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="H63" s="18" t="s">
-        <v>240</v>
+        <v>234</v>
       </c>
       <c r="I63" s="20" t="s">
         <v>36</v>
@@ -8379,7 +8379,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="K63" s="19" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="L63" s="18" t="s">
         <v>36</v>
@@ -8427,7 +8427,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="AA63" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AB63" s="22">
         <v>2</v>
@@ -8464,25 +8464,25 @@
         <v>9960299804</v>
       </c>
       <c r="B64" s="25" t="s">
-        <v>241</v>
+        <v>235</v>
       </c>
       <c r="C64" s="25" t="s">
+        <v>64</v>
+      </c>
+      <c r="D64" s="26" t="s">
         <v>65</v>
       </c>
-      <c r="D64" s="26" t="s">
-        <v>66</v>
-      </c>
       <c r="E64" s="25" t="s">
-        <v>242</v>
+        <v>236</v>
       </c>
       <c r="F64" s="25" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G64" s="26" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H64" s="25" t="s">
-        <v>243</v>
+        <v>237</v>
       </c>
       <c r="I64" s="27" t="s">
         <v>36</v>
@@ -8491,10 +8491,10 @@
         <v>#VALUE!</v>
       </c>
       <c r="K64" s="26" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="L64" s="25" t="s">
-        <v>244</v>
+        <v>238</v>
       </c>
       <c r="M64" s="27" t="s">
         <v>36</v>
@@ -8503,7 +8503,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="O64" s="26" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="P64" s="25" t="s">
         <v>36</v>
@@ -8539,7 +8539,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="AA64" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AB64" s="22">
         <v>2</v>
@@ -8573,7 +8573,7 @@
         <v>9881402331</v>
       </c>
       <c r="B65" s="29" t="s">
-        <v>245</v>
+        <v>239</v>
       </c>
       <c r="C65" s="29" t="s">
         <v>40</v>
@@ -8582,7 +8582,7 @@
         <v>41</v>
       </c>
       <c r="E65" s="29" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
       <c r="F65" s="29" t="s">
         <v>40</v>
@@ -8645,10 +8645,10 @@
         <v>#VALUE!</v>
       </c>
       <c r="Z65" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AA65" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AB65" s="22">
         <v>2</v>
@@ -8682,25 +8682,25 @@
         <v>9822554664</v>
       </c>
       <c r="B66" s="18" t="s">
-        <v>247</v>
+        <v>241</v>
       </c>
       <c r="C66" s="18" t="s">
+        <v>64</v>
+      </c>
+      <c r="D66" s="19" t="s">
         <v>65</v>
       </c>
-      <c r="D66" s="19" t="s">
-        <v>66</v>
-      </c>
       <c r="E66" s="18" t="s">
-        <v>248</v>
+        <v>242</v>
       </c>
       <c r="F66" s="18" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G66" s="19" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H66" s="18" t="s">
-        <v>249</v>
+        <v>243</v>
       </c>
       <c r="I66" s="20" t="s">
         <v>36</v>
@@ -8709,7 +8709,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="K66" s="19" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="L66" s="18" t="s">
         <v>36</v>
@@ -8757,7 +8757,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="AA66" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AB66" s="22">
         <v>2</v>
@@ -8792,7 +8792,7 @@
         <v>9881874309</v>
       </c>
       <c r="B67" s="25" t="s">
-        <v>250</v>
+        <v>244</v>
       </c>
       <c r="C67" s="25" t="s">
         <v>55</v>
@@ -8801,7 +8801,7 @@
         <v>56</v>
       </c>
       <c r="E67" s="25" t="s">
-        <v>251</v>
+        <v>245</v>
       </c>
       <c r="F67" s="25" t="s">
         <v>55</v>
@@ -8810,7 +8810,7 @@
         <v>58</v>
       </c>
       <c r="H67" s="25" t="s">
-        <v>252</v>
+        <v>246</v>
       </c>
       <c r="I67" s="27" t="s">
         <v>36</v>
@@ -8867,7 +8867,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="AA67" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AB67" s="22">
         <v>2</v>
@@ -8891,7 +8891,7 @@
         <v>7700</v>
       </c>
       <c r="AI67" s="22" t="s">
-        <v>253</v>
+        <v>247</v>
       </c>
       <c r="AJ67" s="22">
         <v>1300</v>
@@ -8903,7 +8903,7 @@
         <v>9011033770</v>
       </c>
       <c r="B68" s="29" t="s">
-        <v>254</v>
+        <v>248</v>
       </c>
       <c r="C68" s="29" t="s">
         <v>40</v>
@@ -8912,7 +8912,7 @@
         <v>41</v>
       </c>
       <c r="E68" s="29" t="s">
-        <v>255</v>
+        <v>249</v>
       </c>
       <c r="F68" s="29" t="s">
         <v>40</v>
@@ -8921,7 +8921,7 @@
         <v>43</v>
       </c>
       <c r="H68" s="29" t="s">
-        <v>256</v>
+        <v>250</v>
       </c>
       <c r="I68" s="31" t="s">
         <v>36</v>
@@ -8978,7 +8978,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="AA68" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AB68" s="22">
         <v>2</v>
@@ -9014,25 +9014,25 @@
         <v>9049057671</v>
       </c>
       <c r="B69" s="18" t="s">
-        <v>257</v>
+        <v>251</v>
       </c>
       <c r="C69" s="18">
         <v>9</v>
       </c>
       <c r="D69" s="19" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="E69" s="18" t="s">
-        <v>258</v>
+        <v>252</v>
       </c>
       <c r="F69" s="18">
         <v>8</v>
       </c>
       <c r="G69" s="19" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="H69" s="18" t="s">
-        <v>259</v>
+        <v>253</v>
       </c>
       <c r="I69" s="20" t="s">
         <v>36</v>
@@ -9041,10 +9041,10 @@
         <v>#VALUE!</v>
       </c>
       <c r="K69" s="19" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="L69" s="18" t="s">
-        <v>260</v>
+        <v>254</v>
       </c>
       <c r="M69" s="20" t="s">
         <v>36</v>
@@ -9053,7 +9053,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="O69" s="19" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="P69" s="18" t="s">
         <v>36</v>
@@ -9089,7 +9089,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="AA69" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AB69" s="22">
         <v>2</v>
@@ -9126,7 +9126,7 @@
         <v>9422313106</v>
       </c>
       <c r="B70" s="25" t="s">
-        <v>261</v>
+        <v>255</v>
       </c>
       <c r="C70" s="25" t="s">
         <v>55</v>
@@ -9135,7 +9135,7 @@
         <v>56</v>
       </c>
       <c r="E70" s="25" t="s">
-        <v>262</v>
+        <v>256</v>
       </c>
       <c r="F70" s="25" t="s">
         <v>55</v>
@@ -9144,7 +9144,7 @@
         <v>58</v>
       </c>
       <c r="H70" s="25" t="s">
-        <v>263</v>
+        <v>257</v>
       </c>
       <c r="I70" s="27" t="s">
         <v>36</v>
@@ -9153,7 +9153,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="K70" s="26" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="L70" s="25" t="s">
         <v>36</v>
@@ -9201,7 +9201,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="AA70" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AB70" s="22">
         <v>2</v>
@@ -9221,7 +9221,7 @@
         <v>11400</v>
       </c>
       <c r="AI70" s="22" t="s">
-        <v>264</v>
+        <v>258</v>
       </c>
       <c r="AJ70" s="22">
         <v>0</v>
@@ -9233,25 +9233,25 @@
         <v>9822541922</v>
       </c>
       <c r="B71" s="29" t="s">
-        <v>265</v>
+        <v>259</v>
       </c>
       <c r="C71" s="29">
         <v>9</v>
       </c>
       <c r="D71" s="30" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="E71" s="29" t="s">
-        <v>266</v>
+        <v>260</v>
       </c>
       <c r="F71" s="29">
         <v>8</v>
       </c>
       <c r="G71" s="30" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="H71" s="29" t="s">
-        <v>267</v>
+        <v>261</v>
       </c>
       <c r="I71" s="31" t="s">
         <v>36</v>
@@ -9260,20 +9260,20 @@
         <v>#VALUE!</v>
       </c>
       <c r="K71" s="30" t="s">
+        <v>93</v>
+      </c>
+      <c r="L71" s="29" t="s">
+        <v>262</v>
+      </c>
+      <c r="M71" s="31" t="s">
+        <v>36</v>
+      </c>
+      <c r="N71" s="29" t="e">
+        <v>#VALUE!</v>
+      </c>
+      <c r="O71" s="30" t="s">
         <v>95</v>
       </c>
-      <c r="L71" s="29" t="s">
-        <v>268</v>
-      </c>
-      <c r="M71" s="31" t="s">
-        <v>36</v>
-      </c>
-      <c r="N71" s="29" t="e">
-        <v>#VALUE!</v>
-      </c>
-      <c r="O71" s="30" t="s">
-        <v>97</v>
-      </c>
       <c r="P71" s="29" t="s">
         <v>36</v>
       </c>
@@ -9308,7 +9308,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="AA71" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AB71" s="22">
         <v>2</v>
@@ -9344,25 +9344,25 @@
         <v>9422322202</v>
       </c>
       <c r="B72" s="18" t="s">
-        <v>269</v>
+        <v>263</v>
       </c>
       <c r="C72" s="18">
         <v>3</v>
       </c>
       <c r="D72" s="19" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E72" s="18" t="s">
-        <v>270</v>
+        <v>264</v>
       </c>
       <c r="F72" s="18" t="s">
+        <v>74</v>
+      </c>
+      <c r="G72" s="19" t="s">
         <v>75</v>
       </c>
-      <c r="G72" s="19" t="s">
-        <v>76</v>
-      </c>
       <c r="H72" s="18" t="s">
-        <v>271</v>
+        <v>265</v>
       </c>
       <c r="I72" s="20" t="s">
         <v>36</v>
@@ -9371,7 +9371,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="K72" s="19" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="L72" s="18" t="s">
         <v>36</v>
@@ -9419,7 +9419,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="AA72" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AB72" s="22">
         <v>2</v>
@@ -9458,25 +9458,25 @@
         <v>9420496794</v>
       </c>
       <c r="B73" s="25" t="s">
-        <v>272</v>
+        <v>266</v>
       </c>
       <c r="C73" s="25">
         <v>9</v>
       </c>
       <c r="D73" s="26" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="E73" s="25" t="s">
-        <v>273</v>
+        <v>267</v>
       </c>
       <c r="F73" s="25">
         <v>8</v>
       </c>
       <c r="G73" s="26" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="H73" s="25" t="s">
-        <v>274</v>
+        <v>268</v>
       </c>
       <c r="I73" s="27" t="s">
         <v>36</v>
@@ -9485,10 +9485,10 @@
         <v>#VALUE!</v>
       </c>
       <c r="K73" s="26" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="L73" s="25" t="s">
-        <v>275</v>
+        <v>269</v>
       </c>
       <c r="M73" s="27" t="s">
         <v>36</v>
@@ -9497,7 +9497,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="O73" s="26" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="P73" s="25" t="s">
         <v>36</v>
@@ -9533,7 +9533,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="AA73" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AB73" s="22">
         <v>2</v>
@@ -9571,25 +9571,25 @@
         <v>9860147770</v>
       </c>
       <c r="B74" s="29" t="s">
-        <v>276</v>
+        <v>270</v>
       </c>
       <c r="C74" s="29">
         <v>5</v>
       </c>
       <c r="D74" s="30" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E74" s="29" t="s">
-        <v>277</v>
+        <v>271</v>
       </c>
       <c r="F74" s="29">
         <v>3</v>
       </c>
       <c r="G74" s="30" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="H74" s="29" t="s">
-        <v>278</v>
+        <v>272</v>
       </c>
       <c r="I74" s="31" t="s">
         <v>36</v>
@@ -9598,7 +9598,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="K74" s="30" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="L74" s="29" t="s">
         <v>36</v>
@@ -9646,7 +9646,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="AA74" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AB74" s="22">
         <v>2</v>
@@ -9680,7 +9680,7 @@
         <v>9028847311</v>
       </c>
       <c r="B75" s="18" t="s">
-        <v>279</v>
+        <v>273</v>
       </c>
       <c r="C75" s="18" t="s">
         <v>55</v>
@@ -9689,7 +9689,7 @@
         <v>56</v>
       </c>
       <c r="E75" s="18" t="s">
-        <v>280</v>
+        <v>274</v>
       </c>
       <c r="F75" s="18" t="s">
         <v>55</v>
@@ -9698,7 +9698,7 @@
         <v>58</v>
       </c>
       <c r="H75" s="18" t="s">
-        <v>281</v>
+        <v>275</v>
       </c>
       <c r="I75" s="20" t="s">
         <v>36</v>
@@ -9755,7 +9755,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="AA75" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AB75" s="22">
         <v>2</v>
@@ -9777,7 +9777,7 @@
         <v>10200</v>
       </c>
       <c r="AI75" s="22" t="s">
-        <v>282</v>
+        <v>276</v>
       </c>
       <c r="AJ75" s="22">
         <v>0</v>
@@ -9790,25 +9790,25 @@
         <v>9421011909</v>
       </c>
       <c r="B76" s="25" t="s">
-        <v>283</v>
+        <v>277</v>
       </c>
       <c r="C76" s="25">
         <v>6</v>
       </c>
       <c r="D76" s="26" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="E76" s="25" t="s">
-        <v>284</v>
+        <v>278</v>
       </c>
       <c r="F76" s="25">
         <v>4</v>
       </c>
       <c r="G76" s="26" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="H76" s="25" t="s">
-        <v>285</v>
+        <v>279</v>
       </c>
       <c r="I76" s="27" t="s">
         <v>36</v>
@@ -9817,7 +9817,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="K76" s="26" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="L76" s="25" t="s">
         <v>36</v>
@@ -9865,7 +9865,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="AA76" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AB76" s="22">
         <v>2</v>
@@ -9901,25 +9901,25 @@
         <v>7020629707</v>
       </c>
       <c r="B77" s="29" t="s">
-        <v>286</v>
+        <v>295</v>
       </c>
       <c r="C77" s="29">
         <v>6</v>
       </c>
       <c r="D77" s="30" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="E77" s="29" t="s">
-        <v>287</v>
+        <v>298</v>
       </c>
       <c r="F77" s="29">
         <v>4</v>
       </c>
       <c r="G77" s="30" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="H77" s="29" t="s">
-        <v>288</v>
+        <v>280</v>
       </c>
       <c r="I77" s="31" t="s">
         <v>36</v>
@@ -9928,10 +9928,10 @@
         <v>#VALUE!</v>
       </c>
       <c r="K77" s="30" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="L77" s="29" t="s">
-        <v>289</v>
+        <v>281</v>
       </c>
       <c r="M77" s="31" t="s">
         <v>36</v>
@@ -9940,10 +9940,10 @@
         <v>#VALUE!</v>
       </c>
       <c r="O77" s="30" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="P77" s="29" t="s">
-        <v>290</v>
+        <v>282</v>
       </c>
       <c r="Q77" s="31" t="s">
         <v>36</v>
@@ -9952,10 +9952,10 @@
         <v>#VALUE!</v>
       </c>
       <c r="S77" s="29" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="T77" s="29" t="s">
-        <v>291</v>
+        <v>283</v>
       </c>
       <c r="U77" s="31" t="s">
         <v>36</v>
@@ -9964,7 +9964,7 @@
         <v>36</v>
       </c>
       <c r="W77" s="29" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="X77" s="21" t="e">
         <v>#VALUE!</v>
@@ -9976,7 +9976,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="AA77" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AB77" s="22">
         <v>2</v>
@@ -10014,22 +10014,22 @@
         <v>9021212125</v>
       </c>
       <c r="B78" s="18" t="s">
-        <v>292</v>
+        <v>284</v>
       </c>
       <c r="C78" s="18">
         <v>11</v>
       </c>
       <c r="D78" s="19" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="E78" s="18" t="s">
-        <v>293</v>
+        <v>285</v>
       </c>
       <c r="F78" s="18">
         <v>10</v>
       </c>
       <c r="G78" s="19" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H78" s="18" t="s">
         <v>36</v>
@@ -10086,10 +10086,10 @@
         <v>#VALUE!</v>
       </c>
       <c r="Z78" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AA78" s="21" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AB78" s="22">
         <v>2</v>

</xml_diff>